<commit_message>
- Best LFCC + Delta model so far - Updated the spreadsheet with wav2vec results
</commit_message>
<xml_diff>
--- a/Training_Results_Template_with_Charts.xlsx
+++ b/Training_Results_Template_with_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felip\teamlab-phonetics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45E9BA3-A77A-4B2E-8DD9-6E91C1328FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C753181E-B015-42EC-9B17-BD1774EFD3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>Feature Type</t>
   </si>
@@ -73,9 +73,6 @@
     <t>CNN</t>
   </si>
   <si>
-    <t>Whole dataset</t>
-  </si>
-  <si>
     <t>LogMEL + Δ</t>
   </si>
   <si>
@@ -83,6 +80,18 @@
   </si>
   <si>
     <t>LFCC + Δ</t>
+  </si>
+  <si>
+    <t>EER Training/Validation</t>
+  </si>
+  <si>
+    <t>Less accuracy than the others, but better EER and F1</t>
+  </si>
+  <si>
+    <t>Full dataset</t>
+  </si>
+  <si>
+    <t>v1</t>
   </si>
 </sst>
 </file>
@@ -138,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -149,11 +158,17 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -279,7 +294,10 @@
                   <c:v>10.84</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.2</c:v>
+                  <c:v>6.83</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -490,7 +508,10 @@
                   <c:v>0.62929999999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5978</c:v>
+                  <c:v>0.73</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.79749999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -701,7 +722,10 @@
                   <c:v>53.04</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>62.29</c:v>
+                  <c:v>74.38</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>95.61</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -815,7 +839,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>609599</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -846,7 +870,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -879,7 +903,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -914,10 +938,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:K9" headerRowDxfId="1">
-  <autoFilter ref="A1:K9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="11">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Feature Type" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:L9" headerRowDxfId="2">
+  <autoFilter ref="A1:L9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Feature Type" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Model Architecture"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="# Samples"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Patience"/>
@@ -928,6 +952,7 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="F1 Score"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Accuracy (%)"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Additional Info"/>
+    <tableColumn id="1" xr3:uid="{241E01D4-BC5E-46D0-964C-94B99384C214}" name="EER Training/Validation" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1218,7 +1243,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -1230,10 +1255,10 @@
     <col min="8" max="8" width="15.88671875" customWidth="1"/>
     <col min="9" max="9" width="13.77734375" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="25" customWidth="1"/>
+    <col min="11" max="12" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1267,8 +1292,11 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1282,8 +1310,9 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1297,8 +1326,9 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1312,8 +1342,9 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1321,7 +1352,7 @@
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D5" s="1">
         <v>10</v>
@@ -1345,10 +1376,11 @@
         <v>53.04</v>
       </c>
       <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1360,10 +1392,11 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1375,22 +1408,23 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D8" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E8" s="1">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="F8" s="1">
         <v>64</v>
@@ -1399,30 +1433,58 @@
         <v>1E-4</v>
       </c>
       <c r="H8" s="1">
-        <v>12.2</v>
+        <v>6.83</v>
       </c>
       <c r="I8" s="1">
-        <v>0.5978</v>
+        <v>0.73</v>
       </c>
       <c r="J8" s="1">
-        <v>62.29</v>
-      </c>
-      <c r="K8" s="1"/>
+        <v>74.38</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0.31</v>
+      </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1">
+        <v>28</v>
+      </c>
+      <c r="F9" s="1">
+        <v>64</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1E-4</v>
+      </c>
+      <c r="H9" s="1">
+        <v>4.99</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0.79749999999999999</v>
+      </c>
+      <c r="J9" s="1">
+        <v>95.61</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="1">
+        <v>1.99</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
- Wav2vec V3 Model Weights
</commit_message>
<xml_diff>
--- a/Training_Results_Template_with_Charts.xlsx
+++ b/Training_Results_Template_with_Charts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felip\teamlab-phonetics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Felipe\Team Lab\teamlab-phonetics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C753181E-B015-42EC-9B17-BD1774EFD3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66D880E-5F2E-423F-8C02-CF1E964F76DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
   <si>
     <t>Feature Type</t>
   </si>
@@ -92,6 +92,15 @@
   </si>
   <si>
     <t>v1</t>
+  </si>
+  <si>
+    <t>wav2vec v3</t>
+  </si>
+  <si>
+    <t>Deeper CNN</t>
+  </si>
+  <si>
+    <t>256 h. dimensions / Precision: 0.7413 / Recall: 0.9614</t>
   </si>
 </sst>
 </file>
@@ -147,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -160,6 +169,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -254,9 +266,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Training Results'!$A$2:$A$9</c:f>
+              <c:f>'Training Results'!$A$2:$A$10</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>STFT</c:v>
                 </c:pt>
@@ -280,16 +292,19 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>wav2vec</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>wav2vec v3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Training Results'!$H$2:$H$9</c:f>
+              <c:f>'Training Results'!$H$2:$H$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="3">
                   <c:v>10.84</c:v>
                 </c:pt>
@@ -298,6 +313,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>4.99</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.86</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -468,9 +486,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Training Results'!$A$2:$A$9</c:f>
+              <c:f>'Training Results'!$A$2:$A$10</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>STFT</c:v>
                 </c:pt>
@@ -494,16 +512,19 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>wav2vec</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>wav2vec v3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Training Results'!$I$2:$I$9</c:f>
+              <c:f>'Training Results'!$I$2:$I$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="3">
                   <c:v>0.62929999999999997</c:v>
                 </c:pt>
@@ -512,6 +533,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.79749999999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.83709999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -682,9 +706,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Training Results'!$A$2:$A$9</c:f>
+              <c:f>'Training Results'!$A$2:$A$10</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>STFT</c:v>
                 </c:pt>
@@ -708,16 +732,19 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>wav2vec</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>wav2vec v3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Training Results'!$J$2:$J$9</c:f>
+              <c:f>'Training Results'!$J$2:$J$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="3">
                   <c:v>53.04</c:v>
                 </c:pt>
@@ -726,6 +753,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>95.61</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>96.36</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -938,8 +968,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:L9" headerRowDxfId="2">
-  <autoFilter ref="A1:L9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:L10" headerRowDxfId="2">
+  <autoFilter ref="A1:L10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Feature Type" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Model Architecture"/>
@@ -1243,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -1255,7 +1285,8 @@
     <col min="8" max="8" width="15.88671875" customWidth="1"/>
     <col min="9" max="9" width="13.77734375" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="12" width="25" customWidth="1"/>
+    <col min="11" max="11" width="50.88671875" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -1486,6 +1517,44 @@
         <v>1.99</v>
       </c>
     </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5">
+        <v>5</v>
+      </c>
+      <c r="E10" s="5">
+        <v>18</v>
+      </c>
+      <c r="F10" s="5">
+        <v>64</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1E-4</v>
+      </c>
+      <c r="H10" s="5">
+        <v>3.86</v>
+      </c>
+      <c r="I10" s="5">
+        <v>0.83709999999999996</v>
+      </c>
+      <c r="J10" s="5">
+        <v>96.36</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="1">
+        <v>1.28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>